<commit_message>
updated all the files
</commit_message>
<xml_diff>
--- a/data/Heat map 5.xlsx
+++ b/data/Heat map 5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EAC98E1-615E-400E-A57E-8C9C79BC41AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036980D9-2D3B-42ED-B304-E3691613A516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9DC939E2-9D2B-49F9-96FE-7432C9E71486}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>KPI by Nr.</t>
   </si>
@@ -147,7 +147,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -601,7 +601,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -684,9 +684,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1102,46 +1099,46 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:X26"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="3.21875" style="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.21875" style="14" customWidth="1"/>
-    <col min="4" max="5" width="9.77734375" style="35" customWidth="1"/>
-    <col min="6" max="6" width="9.77734375" style="36" customWidth="1"/>
+    <col min="4" max="5" width="9.77734375" style="34" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" style="35" customWidth="1"/>
     <col min="7" max="11" width="9.77734375" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="15" thickBot="1">
+    <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B1" s="1"/>
-      <c r="C1" s="50" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="53"/>
-    </row>
-    <row r="2" spans="2:11" s="3" customFormat="1" ht="25.95" customHeight="1" thickBot="1">
+      <c r="C1" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="52"/>
+    </row>
+    <row r="2" spans="2:11" s="3" customFormat="1" ht="25.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="2"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="54" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="57" t="s">
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="57"/>
-      <c r="K2" s="58"/>
-    </row>
-    <row r="3" spans="2:11" s="11" customFormat="1" ht="132" customHeight="1" thickBot="1">
+      <c r="J2" s="56"/>
+      <c r="K2" s="57"/>
+    </row>
+    <row r="3" spans="2:11" s="11" customFormat="1" ht="132" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5" t="s">
@@ -1169,8 +1166,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B4" s="47" t="s">
+    <row r="4" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="46" t="s">
         <v>29</v>
       </c>
       <c r="C4" s="15" t="s">
@@ -1188,19 +1185,21 @@
       <c r="G4" s="28">
         <v>0</v>
       </c>
-      <c r="H4" s="29"/>
-      <c r="I4" s="38">
-        <v>0</v>
-      </c>
-      <c r="J4" s="39">
-        <v>0</v>
-      </c>
-      <c r="K4" s="40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B5" s="48"/>
+      <c r="H4" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I4" s="37">
+        <v>0</v>
+      </c>
+      <c r="J4" s="38">
+        <v>0</v>
+      </c>
+      <c r="K4" s="39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="47"/>
       <c r="C5" s="16" t="s">
         <v>5</v>
       </c>
@@ -1216,19 +1215,21 @@
       <c r="G5" s="28">
         <v>3</v>
       </c>
-      <c r="H5" s="29"/>
-      <c r="I5" s="41">
+      <c r="H5" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I5" s="40">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J5" s="42">
+      <c r="J5" s="41">
         <v>0.14000000000000001</v>
       </c>
-      <c r="K5" s="40">
+      <c r="K5" s="39">
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="6" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B6" s="48"/>
+    <row r="6" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="47"/>
       <c r="C6" s="16" t="s">
         <v>6</v>
       </c>
@@ -1244,19 +1245,21 @@
       <c r="G6" s="28">
         <v>1</v>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="41">
-        <v>0</v>
-      </c>
-      <c r="J6" s="42">
-        <v>0</v>
-      </c>
-      <c r="K6" s="43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B7" s="49"/>
+      <c r="H6" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" s="40">
+        <v>0</v>
+      </c>
+      <c r="J6" s="41">
+        <v>0</v>
+      </c>
+      <c r="K6" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="48"/>
       <c r="C7" s="17" t="s">
         <v>7</v>
       </c>
@@ -1272,19 +1275,21 @@
       <c r="G7" s="28">
         <v>0</v>
       </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="44">
+      <c r="H7" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I7" s="43">
         <v>0.43</v>
       </c>
-      <c r="J7" s="45">
+      <c r="J7" s="44">
         <v>0.28999999999999998</v>
       </c>
-      <c r="K7" s="46">
+      <c r="K7" s="45">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="8" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B8" s="47" t="s">
+    <row r="8" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="46" t="s">
         <v>30</v>
       </c>
       <c r="C8" s="15" t="s">
@@ -1302,19 +1307,21 @@
       <c r="G8" s="28">
         <v>5</v>
       </c>
-      <c r="H8" s="29"/>
-      <c r="I8" s="38">
+      <c r="H8" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I8" s="37">
         <v>0.33</v>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="38">
         <v>0.33</v>
       </c>
-      <c r="K8" s="40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B9" s="48"/>
+      <c r="K8" s="39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="47"/>
       <c r="C9" s="16" t="s">
         <v>9</v>
       </c>
@@ -1330,19 +1337,21 @@
       <c r="G9" s="28">
         <v>3</v>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="41">
+      <c r="H9" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I9" s="40">
         <v>0.44</v>
       </c>
-      <c r="J9" s="42">
+      <c r="J9" s="41">
         <v>0.44</v>
       </c>
-      <c r="K9" s="46">
+      <c r="K9" s="45">
         <v>0.11</v>
       </c>
     </row>
-    <row r="10" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B10" s="48"/>
+    <row r="10" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="47"/>
       <c r="C10" s="16" t="s">
         <v>14</v>
       </c>
@@ -1358,19 +1367,21 @@
       <c r="G10" s="28">
         <v>0</v>
       </c>
-      <c r="H10" s="29"/>
-      <c r="I10" s="41">
+      <c r="H10" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I10" s="40">
         <v>0.56999999999999995</v>
       </c>
-      <c r="J10" s="42">
+      <c r="J10" s="41">
         <v>0.71</v>
       </c>
-      <c r="K10" s="43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B11" s="49"/>
+      <c r="K10" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="48"/>
       <c r="C11" s="17" t="s">
         <v>10</v>
       </c>
@@ -1386,19 +1397,21 @@
       <c r="G11" s="28">
         <v>0</v>
       </c>
-      <c r="H11" s="29"/>
-      <c r="I11" s="44">
-        <v>0</v>
-      </c>
-      <c r="J11" s="45">
-        <v>0</v>
-      </c>
-      <c r="K11" s="46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B12" s="47" t="s">
+      <c r="H11" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I11" s="43">
+        <v>0</v>
+      </c>
+      <c r="J11" s="44">
+        <v>0</v>
+      </c>
+      <c r="K11" s="45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="46" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="15" t="s">
@@ -1416,19 +1429,21 @@
       <c r="G12" s="28">
         <v>0</v>
       </c>
-      <c r="H12" s="29"/>
-      <c r="I12" s="38">
-        <v>0</v>
-      </c>
-      <c r="J12" s="39">
-        <v>0</v>
-      </c>
-      <c r="K12" s="40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B13" s="48"/>
+      <c r="H12" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I12" s="37">
+        <v>0</v>
+      </c>
+      <c r="J12" s="38">
+        <v>0</v>
+      </c>
+      <c r="K12" s="39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="47"/>
       <c r="C13" s="16" t="s">
         <v>16</v>
       </c>
@@ -1444,19 +1459,21 @@
       <c r="G13" s="28">
         <v>3</v>
       </c>
-      <c r="H13" s="29"/>
-      <c r="I13" s="41">
-        <v>0</v>
-      </c>
-      <c r="J13" s="42">
-        <v>0</v>
-      </c>
-      <c r="K13" s="43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B14" s="48"/>
+      <c r="H13" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I13" s="40">
+        <v>0</v>
+      </c>
+      <c r="J13" s="41">
+        <v>0</v>
+      </c>
+      <c r="K13" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="47"/>
       <c r="C14" s="16" t="s">
         <v>17</v>
       </c>
@@ -1472,19 +1489,21 @@
       <c r="G14" s="28">
         <v>3</v>
       </c>
-      <c r="H14" s="29"/>
-      <c r="I14" s="41">
-        <v>0</v>
-      </c>
-      <c r="J14" s="42">
-        <v>0</v>
-      </c>
-      <c r="K14" s="43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B15" s="48"/>
+      <c r="H14" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I14" s="40">
+        <v>0</v>
+      </c>
+      <c r="J14" s="41">
+        <v>0</v>
+      </c>
+      <c r="K14" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" s="13" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="47"/>
       <c r="C15" s="16" t="s">
         <v>18</v>
       </c>
@@ -1500,19 +1519,21 @@
       <c r="G15" s="28">
         <v>0</v>
       </c>
-      <c r="H15" s="29"/>
-      <c r="I15" s="41">
-        <v>0</v>
-      </c>
-      <c r="J15" s="42">
-        <v>0</v>
-      </c>
-      <c r="K15" s="43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:11" s="13" customFormat="1" ht="15.45" customHeight="1" thickBot="1">
-      <c r="B16" s="49"/>
+      <c r="H15" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I15" s="40">
+        <v>0</v>
+      </c>
+      <c r="J15" s="41">
+        <v>0</v>
+      </c>
+      <c r="K15" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" s="13" customFormat="1" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="48"/>
       <c r="C16" s="17" t="s">
         <v>19</v>
       </c>
@@ -1528,18 +1549,20 @@
       <c r="G16" s="33">
         <v>0</v>
       </c>
-      <c r="H16" s="34"/>
-      <c r="I16" s="44">
+      <c r="H16" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="I16" s="43">
         <v>1</v>
       </c>
-      <c r="J16" s="45">
-        <v>0</v>
-      </c>
-      <c r="K16" s="46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:24" s="22" customFormat="1" ht="12">
+      <c r="J16" s="44">
+        <v>0</v>
+      </c>
+      <c r="K16" s="45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:24" s="22" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="B17" s="18"/>
       <c r="C17" s="19" t="s">
         <v>11</v>
@@ -1573,7 +1596,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="2:24" s="25" customFormat="1">
+    <row r="18" spans="2:24" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="23"/>
       <c r="C18" s="19" t="s">
         <v>12</v>
@@ -1603,7 +1626,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="19" spans="2:24" s="25" customFormat="1">
+    <row r="19" spans="2:24" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B19" s="23"/>
       <c r="C19" s="19" t="s">
         <v>13</v>
@@ -1650,8 +1673,8 @@
       <c r="W19" s="24"/>
       <c r="X19" s="24"/>
     </row>
-    <row r="26" spans="2:24">
-      <c r="F26" s="36" t="s">
+    <row r="26" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="F26" s="35" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>